<commit_message>
SPM-46: test cases on the fixed seed, 15 -> 14 without overlap
- Merged TC08 (a period covers every slot) into TC09 (it stops on its last
  day): one case on Jurong Expo Floor 16-25 Oct that checks the first day,
  every slot between, and the last day. TC10-TC15 renumbered TC09-TC14.
- Preconditions say the dates are fixed rather than moving with the seed;
  the overlap case says how to restore its data without a reseed.
- Every data-dependent expectation re-checked against the live API on the
  shared database.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-46_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-46_Test_Cases.xlsx
@@ -21,7 +21,6 @@
     <sheet name="TC12" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="TC13" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="TC14" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="TC15" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -461,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -757,7 +756,7 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>A recorded unavailable period covers every slot it spans</t>
+          <t>An unavailable period covers every slot from its first day to its last, and no further</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
@@ -767,7 +766,7 @@
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F11" s="11" t="inlineStr">
@@ -789,17 +788,17 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>A multi-day unavailable period stops on its last day</t>
+          <t>Two overlapping unavailable periods are identified as overlapping</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>AC4</t>
+          <t>AC5</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
@@ -821,12 +820,12 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Two overlapping unavailable periods are identified as overlapping</t>
+          <t>An Event Coordinator and an Operations Manager can open the calendar</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>AC5</t>
+          <t>AC6</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
@@ -853,7 +852,7 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>An Event Coordinator and an Operations Manager can open the calendar</t>
+          <t>A role without venue permissions cannot open the calendar</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -863,7 +862,7 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
@@ -885,17 +884,17 @@
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>A role without venue permissions cannot open the calendar</t>
+          <t>An approved booking blocks its slots, and is listed, even while its event is still in planning</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>AC6</t>
+          <t>AC3, AC7</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr">
@@ -917,17 +916,17 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>An approved booking blocks its slots, and is listed, even while its event is still in planning</t>
+          <t>Only an approved booking takes a slot; a pending request is shown but does not</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>AC3, AC7</t>
+          <t>AC7</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
@@ -949,7 +948,7 @@
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Only an approved booking takes a slot; a pending request is shown but does not</t>
+          <t>A retired venue's slots are never offered as free</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
@@ -968,72 +967,40 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>TC15</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>SPM-46-TC15</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>A retired venue's slots are never offered as free</t>
-        </is>
-      </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>AC7</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>Acceptance Criteria</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Acceptance Criterion</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="9" t="n"/>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Covered by</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="n"/>
+    </row>
+    <row r="21" ht="58" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>AC1</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Users can select a venue and date/time period.</t>
         </is>
       </c>
       <c r="C21" s="8" t="n"/>
       <c r="D21" s="9" t="n"/>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>Covered by</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="n"/>
-    </row>
-    <row r="22" ht="58" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>AC1</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>Users can select a venue and date/time period.</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="11" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>SPM-46-TC01
 SPM-46-TC02
@@ -1041,22 +1008,22 @@
 SPM-46-TC04</t>
         </is>
       </c>
-      <c r="F22" s="9" t="n"/>
-    </row>
-    <row r="23" ht="58" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="F21" s="9" t="n"/>
+    </row>
+    <row r="22" ht="58" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Availability is shown per fixed slot (AM, PM, Night) for each day, including slots occupied by setup or turnaround time.</t>
         </is>
       </c>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>SPM-46-TC01
 SPM-46-TC05
@@ -1064,119 +1031,118 @@
 SPM-46-TC07</t>
         </is>
       </c>
+      <c r="F22" s="9" t="n"/>
+    </row>
+    <row r="23" ht="17.5" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>AC3</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Existing confirmed bookings are displayed.</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>SPM-46-TC12</t>
+        </is>
+      </c>
       <c r="F23" s="9" t="n"/>
     </row>
     <row r="24" ht="17.5" customHeight="1">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>AC3</t>
+          <t>AC4</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Existing confirmed bookings are displayed.</t>
+          <t>Recorded unavailable periods are displayed.</t>
         </is>
       </c>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="9" t="n"/>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>SPM-46-TC13</t>
+          <t>SPM-46-TC08</t>
         </is>
       </c>
       <c r="F24" s="9" t="n"/>
     </row>
-    <row r="25" ht="31" customHeight="1">
+    <row r="25" ht="17.5" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>AC4</t>
+          <t>AC5</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>Recorded unavailable periods are displayed.</t>
+          <t>Overlapping unavailable periods are identifiable.</t>
         </is>
       </c>
       <c r="C25" s="8" t="n"/>
       <c r="D25" s="9" t="n"/>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>SPM-46-TC08
-SPM-46-TC09</t>
+          <t>SPM-46-TC09</t>
         </is>
       </c>
       <c r="F25" s="9" t="n"/>
     </row>
-    <row r="26" ht="17.5" customHeight="1">
+    <row r="26" ht="31" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>AC5</t>
+          <t>AC6</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>Overlapping unavailable periods are identifiable.</t>
+          <t>Only authorised internal users can access the availability calendar.</t>
         </is>
       </c>
       <c r="C26" s="8" t="n"/>
       <c r="D26" s="9" t="n"/>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>SPM-46-TC10</t>
+          <t>SPM-46-TC10
+SPM-46-TC11</t>
         </is>
       </c>
       <c r="F26" s="9" t="n"/>
     </row>
-    <row r="27" ht="31" customHeight="1">
+    <row r="27" ht="44.5" customHeight="1">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>AC6</t>
+          <t>AC7</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>Only authorised internal users can access the availability calendar.</t>
+          <t>Availability reflects confirmed bookings.</t>
         </is>
       </c>
       <c r="C27" s="8" t="n"/>
       <c r="D27" s="9" t="n"/>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>SPM-46-TC11
-SPM-46-TC12</t>
+          <t>SPM-46-TC12
+SPM-46-TC13
+SPM-46-TC14</t>
         </is>
       </c>
       <c r="F27" s="9" t="n"/>
     </row>
-    <row r="28" ht="44.5" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
-        <is>
-          <t>AC7</t>
-        </is>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>Availability reflects confirmed bookings.</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="n"/>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="11" t="inlineStr">
-        <is>
-          <t>SPM-46-TC13
-SPM-46-TC14
-SPM-46-TC15</t>
-        </is>
-      </c>
-      <c r="F28" s="9" t="n"/>
-    </row>
-    <row r="30" ht="125.5" customHeight="1">
-      <c r="A30" s="7" t="inlineStr">
+    <row r="29" ht="125.5" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>Code reviewed</t>
         </is>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>src/app/api/venues/[id]/availability/route.ts
 src/lib/venueAvailability.ts
@@ -1189,17 +1155,18 @@
 design/mockups/VenueCalendar.dc.html</t>
         </is>
       </c>
-      <c r="C30" s="8" t="n"/>
-      <c r="D30" s="8" t="n"/>
-      <c r="E30" s="8" t="n"/>
-      <c r="F30" s="9" t="n"/>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="8" t="n"/>
+      <c r="F29" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="B23:D23"/>
     <mergeCell ref="E24:F24"/>
-    <mergeCell ref="B23:D23"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="E25:F25"/>
     <mergeCell ref="B26:D26"/>
@@ -1209,11 +1176,10 @@
     <mergeCell ref="E22:F22"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B1:F1"/>
-    <mergeCell ref="E28:F28"/>
     <mergeCell ref="E26:F26"/>
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="B24:D24"/>
-    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="B20:D20"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
@@ -1230,7 +1196,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1269,7 +1234,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="112" customHeight="1">
+    <row r="3" ht="166" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1277,13 +1242,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Demo data seeded 2026-09-26 — the dates below move with the seed, because prisma/seed.ts builds them as today + n days (see DOCUMENTATION.md, Known Gaps).
-Marina Boardroom 2 (MAR-BR2) is recorded as unavailable for renovation from 25 Nov 2026 to 9 Dec 2026, ending 23:59 on 9 Dec.
+          <t>Demo data from prisma/seed.ts. Its dates are fixed (2026-09-26 + n days), so a reseed does not move them.
+Jurong Expo Floor (JUR-EXP) has TWO unavailable periods that overlap each other: 'Loading bay hoist inspection.' (maintenance) 5–9 Nov 2026, and 'Fire suppression system recertification.' (safety) 7–11 Nov 2026. They are the only overlapping pair in the demo data — nothing in the app can create one until the Block venue screen (S-23) is built, so they are seeded. If they are missing from the shared database, run: npx tsx prisma/topup-spm40-46.ts (adds them without a reseed).
 Logged in as Venue Staff: marcus.wong@connectsphere.com / password123</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="44.5" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1291,9 +1256,10 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open the availability page for Marina Boardroom 2
-2. Set 'From' to 7 Dec 2026 and 'To' to 13 Dec 2026
-3. Click 'Show availability'</t>
+          <t>1. Open the availability page for Jurong Expo Floor
+2. Set 'From' to 5 Nov 2026 and 'To' to 11 Nov 2026
+3. Click 'Show availability'
+4. Read the 'Unavailable periods' list</t>
         </is>
       </c>
     </row>
@@ -1305,13 +1271,13 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Venue: Marina Boardroom 2 (MAR-BR2)
-From: 7 Dec 2026
-To: 13 Dec 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
+          <t>Venue: Jurong Expo Floor (JUR-EXP)
+From: 5 Nov 2026
+To: 11 Nov 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="98.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1319,7 +1285,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Every slot on 7, 8 and 9 Dec 2026 shows 'Unavailable'. Every slot from 10 to 13 Dec 2026 shows 'Free' — the period stops on its last day and does not spill into 10 Dec. 'Unavailable periods' lists it as 'Refurbishment of the boardroom fit-out.', 25 Nov to 9 Dec 2026.</t>
+          <t>A warning 'Some bookings or unavailable periods overlap' is shown above the grid. Under 'Unavailable periods' both are listed — 'Maintenance', 'Loading bay hoist inspection.' and 'Safety', 'Fire suppression system recertification.' — and EACH carries an 'Overlaps with' note naming the other. Every slot from 5 to 11 Nov 2026 shows 'Unavailable', since between them the two periods cover the whole range.</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1398,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="166" customHeight="1">
+    <row r="3" ht="31" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1440,13 +1406,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Demo data seeded 2026-09-26 — the dates below move with the seed, because prisma/seed.ts builds them as today + n days (see DOCUMENTATION.md, Known Gaps).
-Jurong Expo Floor (JUR-EXP) has TWO unavailable periods that overlap each other: 'Loading bay hoist inspection.' (maintenance) 5–9 Nov 2026, and 'Fire suppression system recertification.' (safety) 7–11 Nov 2026. They are the only overlapping pair in the demo data — nothing in the app can create one until the Block venue screen (S-23) is built, so they are seeded.
-Logged in as Venue Staff: marcus.wong@connectsphere.com / password123</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="58" customHeight="1">
+          <t>Logged in as Event Coordinator: daniel.tan@connectsphere.com / password123</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="85" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1454,10 +1418,10 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open the availability page for Jurong Expo Floor
-2. Set 'From' to 5 Nov 2026 and 'To' to 11 Nov 2026
-3. Click 'Show availability'
-4. Read the 'Unavailable periods' list</t>
+          <t>1. Click 'Venues' in the sidebar
+2. On the 'Marina Grand Hall' row, click 'View availability'
+3. Go back to 'Venues' and click elsewhere on the 'Marina Grand Hall' row
+4. Sign out, sign in as the Operations Manager, and repeat the first two steps</t>
         </is>
       </c>
     </row>
@@ -1469,13 +1433,12 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Venue: Jurong Expo Floor (JUR-EXP)
-From: 5 Nov 2026
-To: 11 Nov 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="98.5" customHeight="1">
+          <t>Accounts: daniel.tan@connectsphere.com (Event Coordinator), grace.lim@connectsphere.com (Operations Manager)
+Venue: Marina Grand Hall (MAR-GH)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="71.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1483,7 +1446,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>A warning 'Some bookings or unavailable periods overlap' is shown above the grid. Under 'Unavailable periods' both are listed — 'Maintenance', 'Loading bay hoist inspection.' and 'Safety', 'Fire suppression system recertification.' — and EACH carries an 'Overlaps with' note naming the other. Every slot from 5 to 11 Nov 2026 shows 'Unavailable', since between them the two periods cover the whole range.</t>
+          <t>Both accounts have 'Venues' in the sidebar, and for both the 'Marina Grand Hall availability' page opens and shows the grid. Clicking elsewhere on the row does nothing — the Venues list stays read-only for both, because neither holds the permission that makes a row editable.</t>
         </is>
       </c>
     </row>
@@ -1596,7 +1559,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="31" customHeight="1">
+    <row r="3" ht="71.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1604,11 +1567,12 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Event Coordinator: daniel.tan@connectsphere.com / password123</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="85" customHeight="1">
+          <t>The tester knows the availability page address for Marina Grand Hall.
+Accounts available: rachel.ng@meridianfina.com (Event Organiser) and kenji.sato@connectsphere.com (Technical Support), both / password123</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1616,14 +1580,16 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Venues' in the sidebar
-2. On the 'Marina Grand Hall' row, click 'View availability'
-3. Go back to 'Venues' and click elsewhere on the 'Marina Grand Hall' row
-4. Sign out, sign in as the Operations Manager, and repeat the first two steps</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44.5" customHeight="1">
+          <t>1. Sign in as the Event Organiser
+2. Confirm there is no 'Venues' item in the sidebar
+3. Paste the Marina Grand Hall availability page address into the address bar and press Enter
+4. Sign out and sign in as Technical Support
+5. Confirm there is no 'Venues' item in their sidebar either
+6. Open the same address again</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1631,12 +1597,12 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Accounts: daniel.tan@connectsphere.com (Event Coordinator), grace.lim@connectsphere.com (Operations Manager)
-Venue: Marina Grand Hall (MAR-GH)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
+          <t>Account: rachel.ng@meridianfina.com (Event Organiser)
+Account: kenji.sato@connectsphere.com (Technical Support)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="166" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1644,7 +1610,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Both accounts have 'Venues' in the sidebar, and for both the 'Marina Grand Hall availability' page opens and shows the grid. Clicking elsewhere on the row does nothing — the Venues list stays read-only for both, because neither holds the permission that makes a row editable.</t>
+          <t>Neither account has 'Venues' in the sidebar, so neither can reach the calendar by navigating — an Event Organiser sees Dashboard, My Events and Notifications; Technical Support sees Dashboard, Equipment, Equipment Requests and Notifications.
+Typing the address directly is refused as well: the page shows 'Venue availability is for ConnectSphere staff', with no grid, no bookings and no unavailable periods. Hiding the link is not the control — the server refuses it too. Technical Support is internal staff and still has no access, because the calendar reuses the venue catalogue's permission, which they do not hold.</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1724,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1765,12 +1732,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>The tester knows the availability page address for Marina Grand Hall.
-Accounts available: rachel.ng@meridianfina.com (Event Organiser) and kenji.sato@connectsphere.com (Technical Support), both / password123</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="98.5" customHeight="1">
+          <t>Demo data from prisma/seed.ts. Its dates are fixed (2026-09-26 + n days), so a reseed does not move them.
+Marina Grand Hall (MAR-GH) has an APPROVED booking, 'Straits Medical Research Symposium', 09:00–18:00 on 7 Dec 2026, whose EVENT is still in Planning — not Confirmed. The venue has a 180-minute setup and 120-minute teardown.
+Logged in as Event Coordinator: daniel.tan@connectsphere.com / password123</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1778,16 +1746,14 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Sign in as the Event Organiser
-2. Confirm there is no 'Venues' item in the sidebar
-3. Paste the Marina Grand Hall availability page address into the address bar and press Enter
-4. Sign out and sign in as Technical Support
-5. Confirm there is no 'Venues' item in their sidebar either
-6. Open the same address again</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
+          <t>1. Open the availability page for Marina Grand Hall
+2. Set 'From' to 6 Dec 2026 and 'To' to 7 Dec 2026
+3. Click 'Show availability'
+4. Read the booking under 'Approved bookings'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1795,12 +1761,13 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Account: rachel.ng@meridianfina.com (Event Organiser)
-Account: kenji.sato@connectsphere.com (Technical Support)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="166" customHeight="1">
+          <t>Venue: Marina Grand Hall (MAR-GH)
+From: 6 Dec 2026
+To: 7 Dec 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="125.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1808,8 +1775,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Neither account has 'Venues' in the sidebar, so neither can reach the calendar by navigating — an Event Organiser sees Dashboard, My Events and Notifications; Technical Support sees Dashboard, Equipment, Equipment Requests and Notifications.
-Typing the address directly is refused as well: the page shows 'Venue availability is for ConnectSphere staff', with no grid, no bookings and no unavailable periods. Hiding the link is not the control — the server refuses it too. Technical Support is internal staff and still has no access, because the calendar reuses the venue catalogue's permission, which they do not hold.</t>
+          <t>On 7 Dec 2026 AM and PM show 'Booked' with 'Straits Medical Research Symposium' — NOT 'Free' — and Night shows 'Turnaround'. On 6 Dec 2026 Night shows 'Turnaround' too, for the setup slot before the event. Under 'Approved bookings' the booking is listed with the event status 'Planning', 7 Dec 2026, 09:00–18:00, layout 'Theatre', and 'Room in use' from 6 Dec 2026, 19:00 to 8 Dec 2026, 00:00. The room must not read as free: an approved booking already commits it, however far its event has got.</t>
         </is>
       </c>
     </row>
@@ -1922,7 +1888,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="125.5" customHeight="1">
+    <row r="3" ht="139" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1930,13 +1896,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Demo data seeded 2026-09-26 — the dates below move with the seed, because prisma/seed.ts builds them as today + n days (see DOCUMENTATION.md, Known Gaps).
-Marina Grand Hall (MAR-GH) has an APPROVED booking, 'Straits Medical Research Symposium', 09:00–18:00 on 7 Dec 2026, whose EVENT is still in Planning — not Confirmed. The venue has a 180-minute setup and 120-minute teardown.
+          <t>Demo data from prisma/seed.ts. Its dates are fixed (2026-09-26 + n days), so a reseed does not move them.
+Changi Conference Centre (CBP-CONF) has a PENDING booking request, 'Pearl Delta Safety Conference', on 14 Dec 2026 and no approved booking that day. Marina Auditorium (MAR-AUD) has a REJECTED booking for 'Nusantara Developer Summit' on 1 Nov 2026. Changi Meeting Room 2 (CBP-MTG2) has a CANCELLED booking for 'Pearl Delta Supplier Forum' on 29 Oct 2026.
 Logged in as Event Coordinator: daniel.tan@connectsphere.com / password123</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="58" customHeight="1">
+    <row r="4" ht="85" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1944,10 +1910,9 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open the availability page for Marina Grand Hall
-2. Set 'From' to 6 Dec 2026 and 'To' to 7 Dec 2026
-3. Click 'Show availability'
-4. Read the booking under 'Approved bookings'</t>
+          <t>1. Open the availability page for Changi Conference Centre for 14 Dec 2026
+2. Choose Marina Auditorium from the 'Venue' picker and show 1 Nov 2026
+3. Choose Changi Meeting Room 2 from the 'Venue' picker and show 29 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -1959,13 +1924,13 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Venue: Marina Grand Hall (MAR-GH)
-From: 6 Dec 2026
-To: 7 Dec 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="125.5" customHeight="1">
+          <t>Changi Conference Centre (CBP-CONF): 14 Dec 2026
+Marina Auditorium (MAR-AUD): 1 Nov 2026
+Changi Meeting Room 2 (CBP-MTG2): 29 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="152.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1973,7 +1938,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>On 7 Dec 2026 AM and PM show 'Booked' with 'Straits Medical Research Symposium' — NOT 'Free' — and Night shows 'Turnaround'. On 6 Dec 2026 Night shows 'Turnaround' too, for the setup slot before the event. Under 'Approved bookings' the booking is listed with the event status 'Planning', 7 Dec 2026, 09:00–18:00, layout 'Theatre', and 'Room in use' from 6 Dec 2026, 19:00 to 8 Dec 2026, 00:00. The room must not read as free: an approved booking already commits it, however far its event has got.</t>
+          <t>On all three days every slot shows 'Free'. None of 'Pearl Delta Safety Conference', 'Nusantara Developer Summit' or 'Pearl Delta Supplier Forum' appears under 'Approved bookings' — only an approved booking takes a room.
+On 14 Dec 2026 the Changi Conference Centre slots additionally carry the note 'Requested: Pearl Delta Safety Conference', and a card 'Requested, not yet approved' lists it below the grid. The slots stay 'Free' — a request is not a commitment — but the hold is visible so a second coordinator does not request the same room unaware. The rejected and cancelled bookings carry no such note: they are not live requests.</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2052,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="152.5" customHeight="1">
+    <row r="3" ht="71.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2094,171 +2060,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Demo data seeded 2026-09-26 — the dates below move with the seed, because prisma/seed.ts builds them as today + n days (see DOCUMENTATION.md, Known Gaps).
-Changi Conference Centre (CBP-CONF) has a PENDING booking request, 'Pearl Delta Safety Conference', on 14 Dec 2026 and no approved booking that day. Marina Auditorium (MAR-AUD) has a REJECTED booking for 'Nusantara Developer Summit' on 1 Nov 2026. Changi Meeting Room 2 (CBP-MTG2) has a CANCELLED booking for 'Pearl Delta Supplier Forum' on 29 Oct 2026.
-Logged in as Event Coordinator: daniel.tan@connectsphere.com / password123</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="85" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Open the availability page for Changi Conference Centre for 14 Dec 2026
-2. Choose Marina Auditorium from the 'Venue' picker and show 1 Nov 2026
-3. Choose Changi Meeting Room 2 from the 'Venue' picker and show 29 Oct 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Changi Conference Centre (CBP-CONF): 14 Dec 2026
-Marina Auditorium (MAR-AUD): 1 Nov 2026
-Changi Meeting Room 2 (CBP-MTG2): 29 Oct 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="152.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>On all three days every slot shows 'Free'. None of 'Pearl Delta Safety Conference', 'Nusantara Developer Summit' or 'Pearl Delta Supplier Forum' appears under 'Approved bookings' — only an approved booking takes a room.
-On 14 Dec 2026 the Changi Conference Centre slots additionally carry the note 'Requested: Pearl Delta Safety Conference', and a card 'Requested, not yet approved' lists it below the grid. The slots stay 'Free' — a request is not a commitment — but the hold is visible so a second coordinator does not request the same room unaware. The rejected and cancelled bookings carry no such note: they are not live requests.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>kayalvizhi24</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-46-TC15</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="85" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Demo data seeded 2026-09-26 — the dates below move with the seed, because prisma/seed.ts builds them as today + n days (see DOCUMENTATION.md, Known Gaps).
+          <t>Demo data from prisma/seed.ts. Its dates are fixed (2026-09-26 + n days), so a reseed does not move them.
 Jurong Skills Lab (JUR-LAB) is active and has no bookings.
 Logged in as Venue Staff: marcus.wong@connectsphere.com / password123</t>
         </is>
@@ -2415,7 +2217,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2423,7 +2225,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Demo data seeded 2026-09-26 — the dates below move with the seed, because prisma/seed.ts builds them as today + n days (see DOCUMENTATION.md, Known Gaps).
+          <t>Demo data from prisma/seed.ts. Its dates are fixed (2026-09-26 + n days), so a reseed does not move them.
 Logged in as Venue Staff: marcus.wong@connectsphere.com / password123</t>
         </is>
       </c>
@@ -2905,7 +2707,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="85" customHeight="1">
+    <row r="3" ht="71.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2913,7 +2715,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Demo data seeded 2026-09-26 — the dates below move with the seed, because prisma/seed.ts builds them as today + n days (see DOCUMENTATION.md, Known Gaps).
+          <t>Demo data from prisma/seed.ts. Its dates are fixed (2026-09-26 + n days), so a reseed does not move them.
 Logged in as Venue Staff: marcus.wong@connectsphere.com / password123
 Viewing Marina Grand Hall's availability for 7–13 Dec 2026.</t>
         </is>
@@ -3065,7 +2867,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="112" customHeight="1">
+    <row r="3" ht="98.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3073,7 +2875,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Demo data seeded 2026-09-26 — the dates below move with the seed, because prisma/seed.ts builds them as today + n days (see DOCUMENTATION.md, Known Gaps).
+          <t>Demo data from prisma/seed.ts. Its dates are fixed (2026-09-26 + n days), so a reseed does not move them.
 One-North Auditorium (ONE-AUD) records setup and teardown time, and has an approved booking, 'Bayu Energy Transition Panel', 18:00–21:00 on 9 Nov 2026.
 Logged in as Venue Staff: marcus.wong@connectsphere.com / password123</t>
         </is>
@@ -3228,7 +3030,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="112" customHeight="1">
+    <row r="3" ht="98.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3236,7 +3038,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Demo data seeded 2026-09-26 — the dates below move with the seed, because prisma/seed.ts builds them as today + n days (see DOCUMENTATION.md, Known Gaps).
+          <t>Demo data from prisma/seed.ts. Its dates are fixed (2026-09-26 + n days), so a reseed does not move them.
 Jurong Expo Floor (JUR-EXP) records setup and teardown time, and has an approved booking, 'Sundara Hospitality Trade Showcase', 10:00–18:00 on 30 Nov 2026.
 Logged in as Venue Staff: marcus.wong@connectsphere.com / password123</t>
         </is>
@@ -3391,7 +3193,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="98.5" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3399,7 +3201,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Demo data seeded 2026-09-26 — the dates below move with the seed, because prisma/seed.ts builds them as today + n days (see DOCUMENTATION.md, Known Gaps).
+          <t>Demo data from prisma/seed.ts. Its dates are fixed (2026-09-26 + n days), so a reseed does not move them.
 One-North Rooftop Terrace (ONE-ROOF) is open 16:00–23:00 only, and has no bookings on this date.
 Logged in as Venue Staff: marcus.wong@connectsphere.com / password123</t>
         </is>
@@ -3554,7 +3356,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="98.5" customHeight="1">
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3562,13 +3364,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Demo data seeded 2026-09-26 — the dates below move with the seed, because prisma/seed.ts builds them as today + n days (see DOCUMENTATION.md, Known Gaps).
-Jurong Expo Floor (JUR-EXP) is recorded as unavailable for renovation from 17 Oct 2026 to 24 Oct 2026.
+          <t>Demo data from prisma/seed.ts. Its dates are fixed (2026-09-26 + n days), so a reseed does not move them.
+Jurong Expo Floor (JUR-EXP) is recorded as unavailable for renovation from 17 Oct 2026, 00:00 to 24 Oct 2026, 23:59, and has nothing else from 16 to 25 Oct 2026. It is open 06:00–23:00.
 Logged in as Venue Staff: marcus.wong@connectsphere.com / password123</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="44.5" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3577,8 +3379,9 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Open the availability page for Jurong Expo Floor
-2. Set 'From' to 17 Oct 2026 and 'To' to 23 Oct 2026
-3. Click 'Show availability'</t>
+2. Set 'From' to 16 Oct 2026 and 'To' to 25 Oct 2026
+3. Click 'Show availability'
+4. Read the 'Unavailable periods' list</t>
         </is>
       </c>
     </row>
@@ -3591,12 +3394,12 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Venue: Jurong Expo Floor (JUR-EXP)
-From: 17 Oct 2026
-To: 23 Oct 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="85" customHeight="1">
+From: 16 Oct 2026
+To: 25 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="125.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3604,7 +3407,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Every slot on every day from 17 to 23 Oct 2026 shows 'Unavailable' — 21 cells, none of them 'Free'. Under 'Unavailable periods' one period is listed: 'Renovation', 'Floor resurfacing and loading bay works.', 17 Oct 2026 to 24 Oct 2026, with no 'Overlaps with' note and no overlap warning above the grid.</t>
+          <t>16 Oct 2026: AM, PM and Night all show 'Free' (Night with the note 'Open until 23:00') — the period does not start early. 17 to 24 Oct 2026: every slot shows 'Unavailable' — 24 cells, none of them 'Free'. 25 Oct 2026: AM, PM and Night all show 'Free' again — the period stops on its last day and does not spill into the next. Under 'Unavailable periods' exactly one period is listed: 'Renovation', 'Floor resurfacing and loading bay works.', 17 Oct 2026 to 24 Oct 2026, with no 'Overlaps with' note and no overlap warning above the grid.</t>
         </is>
       </c>
     </row>

</xml_diff>